<commit_message>
v0.9 errata: workbook boundary notes and simplified platform inputs
</commit_message>
<xml_diff>
--- a/AI_Business_Case_Model.xlsx
+++ b/AI_Business_Case_Model.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Yaroslav\Documents\GitHub\AI-Workbook\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6FAFCC0-226F-44BB-A614-89EFD0FE83A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA79E95F-AD5F-4A7C-9CF4-3A162FD44716}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="23380" yWindow="0" windowWidth="26460" windowHeight="20970" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="23380" yWindow="0" windowWidth="26460" windowHeight="20970" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Read me" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="179" uniqueCount="156">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="154">
   <si>
     <t>AI business case model</t>
   </si>
@@ -483,18 +483,6 @@
     <t>k/month</t>
   </si>
   <si>
-    <t>The monthly cost of the AI-platform specific layer</t>
-  </si>
-  <si>
-    <t>Platform, months charged</t>
-  </si>
-  <si>
-    <t>months</t>
-  </si>
-  <si>
-    <t>Reduce for a mid-year start</t>
-  </si>
-  <si>
     <t>Phase 0 remediation, one-off</t>
   </si>
   <si>
@@ -514,6 +502,12 @@
   </si>
   <si>
     <t>k</t>
+  </si>
+  <si>
+    <t>Net benefit is payroll-equivalent, priced at loaded engineering cost. What finance recognises depends on the conversion route (Section 12)</t>
+  </si>
+  <si>
+    <t>The monthly cost of the AI-specific platform layer.</t>
   </si>
 </sst>
 </file>
@@ -1163,8 +1157,6 @@
     <xf numFmtId="166" fontId="1" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="3" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -1232,6 +1224,84 @@
     <xf numFmtId="166" fontId="3" fillId="7" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="11" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="168" fontId="11" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="12" fillId="5" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="11" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="12" fillId="5" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="11" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="38" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -1269,84 +1339,8 @@
     <xf numFmtId="166" fontId="1" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="11" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="168" fontId="11" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="12" fillId="5" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="11" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="12" fillId="5" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="11" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="38" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="3" fontId="6" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2026,162 +2020,162 @@
   <dimension ref="A2:C33"/>
   <sheetFormatPr defaultColWidth="14.453125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="2" style="31" customWidth="1"/>
-    <col min="2" max="2" width="33.90625" style="31" customWidth="1"/>
-    <col min="3" max="3" width="108.54296875" style="31" customWidth="1"/>
-    <col min="4" max="5" width="14" style="31" customWidth="1"/>
-    <col min="6" max="6" width="8.7265625" style="31" customWidth="1"/>
-    <col min="7" max="7" width="11.453125" style="31" customWidth="1"/>
-    <col min="8" max="16384" width="14.453125" style="31"/>
+    <col min="1" max="1" width="2" style="29" customWidth="1"/>
+    <col min="2" max="2" width="33.90625" style="29" customWidth="1"/>
+    <col min="3" max="3" width="108.54296875" style="29" customWidth="1"/>
+    <col min="4" max="5" width="14" style="29" customWidth="1"/>
+    <col min="6" max="6" width="8.7265625" style="29" customWidth="1"/>
+    <col min="7" max="7" width="11.453125" style="29" customWidth="1"/>
+    <col min="8" max="16384" width="14.453125" style="29"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:3" ht="13" x14ac:dyDescent="0.3">
-      <c r="B2" s="30" t="s">
+      <c r="B2" s="28" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="3" spans="2:3" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="B3" s="32" t="s">
+      <c r="B3" s="30" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="4" spans="2:3" ht="12.5" x14ac:dyDescent="0.25">
-      <c r="B4" s="32" t="s">
+      <c r="B4" s="30" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="6" spans="2:3" ht="37.5" x14ac:dyDescent="0.25">
-      <c r="B6" s="28" t="s">
+      <c r="B6" s="26" t="s">
         <v>3</v>
       </c>
-      <c r="C6" s="29" t="s">
+      <c r="C6" s="27" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="8" spans="2:3" ht="13" x14ac:dyDescent="0.25">
-      <c r="B8" s="28" t="s">
+      <c r="B8" s="26" t="s">
         <v>5</v>
       </c>
-      <c r="C8" s="29" t="s">
+      <c r="C8" s="27" t="s">
         <v>140</v>
       </c>
     </row>
     <row r="10" spans="2:3" ht="25" x14ac:dyDescent="0.25">
-      <c r="B10" s="28" t="s">
+      <c r="B10" s="26" t="s">
         <v>6</v>
       </c>
-      <c r="C10" s="29" t="s">
+      <c r="C10" s="27" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="12" spans="2:3" ht="62.5" x14ac:dyDescent="0.25">
-      <c r="B12" s="28" t="s">
+      <c r="B12" s="26" t="s">
         <v>8</v>
       </c>
-      <c r="C12" s="29" t="s">
+      <c r="C12" s="27" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="14" spans="2:3" ht="62.5" x14ac:dyDescent="0.25">
-      <c r="B14" s="28" t="s">
+      <c r="B14" s="26" t="s">
         <v>10</v>
       </c>
-      <c r="C14" s="29" t="s">
-        <v>154</v>
+      <c r="C14" s="27" t="s">
+        <v>150</v>
       </c>
     </row>
     <row r="16" spans="2:3" ht="13" x14ac:dyDescent="0.25">
-      <c r="B16" s="28" t="s">
+      <c r="B16" s="26" t="s">
         <v>11</v>
       </c>
-      <c r="C16" s="33" t="s">
+      <c r="C16" s="31" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="20" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B20" s="34" t="s">
+      <c r="B20" s="32" t="s">
         <v>141</v>
       </c>
-      <c r="C20" s="34" t="s">
+      <c r="C20" s="32" t="s">
         <v>128</v>
       </c>
     </row>
     <row r="21" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B21" s="35" t="s">
+      <c r="B21" s="33" t="s">
         <v>138</v>
       </c>
-      <c r="C21" s="35" t="s">
+      <c r="C21" s="33" t="s">
         <v>129</v>
       </c>
     </row>
     <row r="22" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B22" s="35" t="s">
+      <c r="B22" s="33" t="s">
         <v>130</v>
       </c>
-      <c r="C22" s="35" t="s">
+      <c r="C22" s="33" t="s">
         <v>142</v>
       </c>
     </row>
     <row r="23" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B23" s="35" t="s">
+      <c r="B23" s="33" t="s">
         <v>131</v>
       </c>
-      <c r="C23" s="35" t="s">
+      <c r="C23" s="33" t="s">
         <v>139</v>
       </c>
     </row>
     <row r="24" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B24" s="35" t="s">
+      <c r="B24" s="33" t="s">
         <v>132</v>
       </c>
-      <c r="C24" s="35" t="s">
+      <c r="C24" s="33" t="s">
         <v>133</v>
       </c>
     </row>
     <row r="25" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="35"/>
-      <c r="B25" s="35" t="s">
+      <c r="A25" s="33"/>
+      <c r="B25" s="33" t="s">
         <v>134</v>
       </c>
-      <c r="C25" s="35" t="s">
+      <c r="C25" s="33" t="s">
         <v>135</v>
       </c>
     </row>
     <row r="26" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B26" s="35" t="s">
+      <c r="B26" s="33" t="s">
         <v>136</v>
       </c>
-      <c r="C26" s="35" t="s">
+      <c r="C26" s="33" t="s">
         <v>137</v>
       </c>
     </row>
     <row r="27" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B27" s="36"/>
-      <c r="C27" s="36"/>
+      <c r="B27" s="34"/>
+      <c r="C27" s="34"/>
     </row>
     <row r="28" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B28" s="36"/>
-      <c r="C28" s="36"/>
+      <c r="B28" s="34"/>
+      <c r="C28" s="34"/>
     </row>
     <row r="29" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B29" s="36"/>
-      <c r="C29" s="36"/>
+      <c r="B29" s="34"/>
+      <c r="C29" s="34"/>
     </row>
     <row r="30" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B30" s="36"/>
-      <c r="C30" s="36"/>
+      <c r="B30" s="34"/>
+      <c r="C30" s="34"/>
     </row>
     <row r="31" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B31" s="36"/>
-      <c r="C31" s="36"/>
+      <c r="B31" s="34"/>
+      <c r="C31" s="34"/>
     </row>
     <row r="32" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B32" s="36"/>
-      <c r="C32" s="36"/>
+      <c r="B32" s="34"/>
+      <c r="C32" s="34"/>
     </row>
     <row r="33" spans="2:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B33" s="36"/>
-      <c r="C33" s="36"/>
+      <c r="B33" s="34"/>
+      <c r="C33" s="34"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
@@ -2191,7 +2185,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="B2:G16"/>
+  <dimension ref="B2:G15"/>
   <sheetFormatPr defaultColWidth="14.453125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="2" customWidth="1"/>
@@ -2206,297 +2200,281 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="63" t="s">
+      <c r="B2" s="46" t="s">
         <v>13</v>
       </c>
-      <c r="C2" s="64" t="s">
+      <c r="C2" s="47" t="s">
         <v>14</v>
       </c>
-      <c r="D2" s="64" t="s">
+      <c r="D2" s="47" t="s">
         <v>15</v>
       </c>
-      <c r="E2" s="64" t="s">
+      <c r="E2" s="47" t="s">
         <v>16</v>
       </c>
-      <c r="F2" s="64" t="s">
+      <c r="F2" s="47" t="s">
         <v>17</v>
       </c>
-      <c r="G2" s="64" t="s">
+      <c r="G2" s="47" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="3" spans="2:7" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B3" s="65" t="s">
+      <c r="B3" s="48" t="s">
         <v>20</v>
       </c>
-      <c r="C3" s="66">
+      <c r="C3" s="49">
         <v>300</v>
       </c>
-      <c r="D3" s="67" t="s">
+      <c r="D3" s="50" t="s">
         <v>23</v>
       </c>
-      <c r="E3" s="68" t="s">
+      <c r="E3" s="51" t="s">
         <v>25</v>
       </c>
-      <c r="F3" s="68" t="s">
+      <c r="F3" s="51" t="s">
         <v>26</v>
       </c>
-      <c r="G3" s="68" t="s">
+      <c r="G3" s="51" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="4" spans="2:7" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B4" s="69" t="s">
+      <c r="B4" s="52" t="s">
         <v>29</v>
       </c>
-      <c r="C4" s="70">
+      <c r="C4" s="53">
         <v>160</v>
       </c>
-      <c r="D4" s="71" t="s">
+      <c r="D4" s="54" t="s">
         <v>31</v>
       </c>
-      <c r="E4" s="72" t="s">
+      <c r="E4" s="55" t="s">
         <v>32</v>
       </c>
-      <c r="F4" s="72" t="s">
+      <c r="F4" s="55" t="s">
         <v>33</v>
       </c>
-      <c r="G4" s="72" t="s">
+      <c r="G4" s="55" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="5" spans="2:7" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B5" s="69" t="s">
+      <c r="B5" s="52" t="s">
         <v>35</v>
       </c>
-      <c r="C5" s="73">
+      <c r="C5" s="56">
         <v>1.25</v>
       </c>
-      <c r="D5" s="71" t="s">
+      <c r="D5" s="54" t="s">
         <v>36</v>
       </c>
-      <c r="E5" s="72" t="s">
+      <c r="E5" s="55" t="s">
         <v>37</v>
       </c>
-      <c r="F5" s="72"/>
-      <c r="G5" s="72" t="s">
+      <c r="F5" s="55"/>
+      <c r="G5" s="55" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="6" spans="2:7" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B6" s="74" t="s">
+      <c r="B6" s="57" t="s">
         <v>40</v>
       </c>
-      <c r="C6" s="75">
+      <c r="C6" s="58">
         <f>400/C5</f>
         <v>320</v>
       </c>
-      <c r="D6" s="76" t="s">
+      <c r="D6" s="59" t="s">
         <v>42</v>
       </c>
-      <c r="E6" s="77" t="s">
+      <c r="E6" s="60" t="s">
         <v>44</v>
       </c>
-      <c r="F6" s="77" t="s">
+      <c r="F6" s="60" t="s">
         <v>46</v>
       </c>
-      <c r="G6" s="77" t="s">
+      <c r="G6" s="60" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="7" spans="2:7" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B7" s="74" t="s">
+      <c r="B7" s="57" t="s">
         <v>48</v>
       </c>
-      <c r="C7" s="78">
+      <c r="C7" s="61">
         <v>60</v>
       </c>
-      <c r="D7" s="76" t="s">
+      <c r="D7" s="59" t="s">
         <v>49</v>
       </c>
-      <c r="E7" s="77" t="s">
+      <c r="E7" s="60" t="s">
         <v>50</v>
       </c>
-      <c r="F7" s="77" t="s">
+      <c r="F7" s="60" t="s">
         <v>51</v>
       </c>
-      <c r="G7" s="77" t="s">
+      <c r="G7" s="60" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="8" spans="2:7" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B8" s="69" t="s">
+      <c r="B8" s="52" t="s">
         <v>57</v>
       </c>
-      <c r="C8" s="79">
+      <c r="C8" s="62">
         <v>3</v>
       </c>
-      <c r="D8" s="71" t="s">
+      <c r="D8" s="54" t="s">
         <v>49</v>
       </c>
-      <c r="E8" s="72" t="s">
+      <c r="E8" s="55" t="s">
         <v>59</v>
       </c>
-      <c r="F8" s="72" t="s">
+      <c r="F8" s="55" t="s">
         <v>60</v>
       </c>
-      <c r="G8" s="72" t="s">
+      <c r="G8" s="55" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="9" spans="2:7" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B9" s="69" t="s">
+      <c r="B9" s="52" t="s">
         <v>62</v>
       </c>
-      <c r="C9" s="79">
+      <c r="C9" s="62">
         <v>2</v>
       </c>
-      <c r="D9" s="71" t="s">
+      <c r="D9" s="54" t="s">
         <v>49</v>
       </c>
-      <c r="E9" s="72" t="s">
+      <c r="E9" s="55" t="s">
         <v>64</v>
       </c>
-      <c r="F9" s="72" t="s">
+      <c r="F9" s="55" t="s">
         <v>65</v>
       </c>
-      <c r="G9" s="72" t="s">
+      <c r="G9" s="55" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="10" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B10" s="80" t="s">
+      <c r="B10" s="63" t="s">
         <v>143</v>
       </c>
-      <c r="C10" s="81">
+      <c r="C10" s="64">
         <v>6</v>
       </c>
-      <c r="D10" s="82" t="s">
+      <c r="D10" s="65" t="s">
         <v>144</v>
       </c>
-      <c r="E10" s="83" t="s">
+      <c r="E10" s="66" t="s">
+        <v>153</v>
+      </c>
+      <c r="F10" s="29"/>
+      <c r="G10" s="66" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="11" spans="2:7" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B11" s="52" t="s">
+        <v>67</v>
+      </c>
+      <c r="C11" s="67">
+        <f>C10*12</f>
+        <v>72</v>
+      </c>
+      <c r="D11" s="54" t="s">
+        <v>31</v>
+      </c>
+      <c r="E11" s="55" t="s">
+        <v>68</v>
+      </c>
+      <c r="F11" s="55" t="s">
+        <v>69</v>
+      </c>
+      <c r="G11" s="55" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="12" spans="2:7" ht="61.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B12" s="57" t="s">
+        <v>72</v>
+      </c>
+      <c r="C12" s="68">
+        <v>1.7</v>
+      </c>
+      <c r="D12" s="59" t="s">
+        <v>73</v>
+      </c>
+      <c r="E12" s="55" t="s">
+        <v>74</v>
+      </c>
+      <c r="F12" s="60" t="s">
+        <v>75</v>
+      </c>
+      <c r="G12" s="60" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="13" spans="2:7" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B13" s="52" t="s">
+        <v>77</v>
+      </c>
+      <c r="C13" s="68">
+        <v>0.8</v>
+      </c>
+      <c r="D13" s="54" t="s">
+        <v>73</v>
+      </c>
+      <c r="E13" s="55" t="s">
+        <v>78</v>
+      </c>
+      <c r="F13" s="55" t="s">
+        <v>79</v>
+      </c>
+      <c r="G13" s="55" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="14" spans="2:7" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B14" s="57" t="s">
+        <v>82</v>
+      </c>
+      <c r="C14" s="64">
+        <v>0</v>
+      </c>
+      <c r="D14" s="59" t="s">
+        <v>31</v>
+      </c>
+      <c r="E14" s="60" t="s">
+        <v>83</v>
+      </c>
+      <c r="F14" s="60" t="s">
+        <v>84</v>
+      </c>
+      <c r="G14" s="60" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="15" spans="2:7" ht="25" x14ac:dyDescent="0.35">
+      <c r="B15" s="52" t="s">
         <v>145</v>
       </c>
-      <c r="F10" s="31"/>
-      <c r="G10" s="83" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="11" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B11" s="69" t="s">
+      <c r="C15" s="53">
+        <v>0</v>
+      </c>
+      <c r="D15" s="54" t="s">
+        <v>151</v>
+      </c>
+      <c r="E15" s="55" t="s">
         <v>146</v>
       </c>
-      <c r="C11" s="79">
-        <v>12</v>
-      </c>
-      <c r="D11" s="71" t="s">
+      <c r="F15" s="55" t="s">
+        <v>148</v>
+      </c>
+      <c r="G15" s="55" t="s">
         <v>147</v>
-      </c>
-      <c r="E11" s="72" t="s">
-        <v>148</v>
-      </c>
-      <c r="F11" s="72"/>
-      <c r="G11" s="72"/>
-    </row>
-    <row r="12" spans="2:7" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B12" s="69" t="s">
-        <v>67</v>
-      </c>
-      <c r="C12" s="84">
-        <f>C10*C11</f>
-        <v>72</v>
-      </c>
-      <c r="D12" s="71" t="s">
-        <v>31</v>
-      </c>
-      <c r="E12" s="72" t="s">
-        <v>68</v>
-      </c>
-      <c r="F12" s="72" t="s">
-        <v>69</v>
-      </c>
-      <c r="G12" s="72" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="13" spans="2:7" ht="61.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B13" s="74" t="s">
-        <v>72</v>
-      </c>
-      <c r="C13" s="85">
-        <v>1.7</v>
-      </c>
-      <c r="D13" s="76" t="s">
-        <v>73</v>
-      </c>
-      <c r="E13" s="72" t="s">
-        <v>74</v>
-      </c>
-      <c r="F13" s="77" t="s">
-        <v>75</v>
-      </c>
-      <c r="G13" s="77" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="14" spans="2:7" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B14" s="69" t="s">
-        <v>77</v>
-      </c>
-      <c r="C14" s="85">
-        <v>0.8</v>
-      </c>
-      <c r="D14" s="71" t="s">
-        <v>73</v>
-      </c>
-      <c r="E14" s="72" t="s">
-        <v>78</v>
-      </c>
-      <c r="F14" s="72" t="s">
-        <v>79</v>
-      </c>
-      <c r="G14" s="72" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="15" spans="2:7" ht="45.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B15" s="74" t="s">
-        <v>82</v>
-      </c>
-      <c r="C15" s="81">
-        <v>0</v>
-      </c>
-      <c r="D15" s="76" t="s">
-        <v>31</v>
-      </c>
-      <c r="E15" s="77" t="s">
-        <v>83</v>
-      </c>
-      <c r="F15" s="77" t="s">
-        <v>84</v>
-      </c>
-      <c r="G15" s="77" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="16" spans="2:7" ht="25" x14ac:dyDescent="0.35">
-      <c r="B16" s="69" t="s">
-        <v>149</v>
-      </c>
-      <c r="C16" s="70">
-        <v>0</v>
-      </c>
-      <c r="D16" s="71" t="s">
-        <v>155</v>
-      </c>
-      <c r="E16" s="72" t="s">
-        <v>150</v>
-      </c>
-      <c r="F16" s="72" t="s">
-        <v>152</v>
-      </c>
-      <c r="G16" s="72" t="s">
-        <v>151</v>
       </c>
     </row>
   </sheetData>
@@ -2513,43 +2491,43 @@
   <dimension ref="B2:K10"/>
   <sheetFormatPr defaultColWidth="14.453125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="1.54296875" style="45" customWidth="1"/>
-    <col min="2" max="2" width="18.7265625" style="45" customWidth="1"/>
-    <col min="3" max="10" width="14.453125" style="45"/>
-    <col min="11" max="11" width="13.54296875" style="45" customWidth="1"/>
-    <col min="12" max="16384" width="14.453125" style="45"/>
+    <col min="1" max="1" width="1.54296875" style="43" customWidth="1"/>
+    <col min="2" max="2" width="18.7265625" style="43" customWidth="1"/>
+    <col min="3" max="10" width="14.453125" style="43"/>
+    <col min="11" max="11" width="13.54296875" style="43" customWidth="1"/>
+    <col min="12" max="16384" width="14.453125" style="43"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:11" ht="32.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="48" t="s">
+      <c r="B2" s="72" t="s">
         <v>27</v>
       </c>
-      <c r="C2" s="49"/>
-      <c r="D2" s="49"/>
-      <c r="E2" s="49"/>
-      <c r="F2" s="49"/>
-      <c r="G2" s="49"/>
-      <c r="H2" s="49"/>
-      <c r="I2" s="49"/>
-      <c r="J2" s="49"/>
-      <c r="K2" s="49"/>
+      <c r="C2" s="73"/>
+      <c r="D2" s="73"/>
+      <c r="E2" s="73"/>
+      <c r="F2" s="73"/>
+      <c r="G2" s="73"/>
+      <c r="H2" s="73"/>
+      <c r="I2" s="73"/>
+      <c r="J2" s="73"/>
+      <c r="K2" s="73"/>
     </row>
     <row r="4" spans="2:11" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="C4" s="50" t="s">
+      <c r="C4" s="74" t="s">
         <v>41</v>
       </c>
-      <c r="D4" s="49"/>
-      <c r="E4" s="49"/>
-      <c r="F4" s="50" t="s">
+      <c r="D4" s="73"/>
+      <c r="E4" s="73"/>
+      <c r="F4" s="74" t="s">
         <v>43</v>
       </c>
-      <c r="G4" s="49"/>
-      <c r="H4" s="49"/>
-      <c r="I4" s="50" t="s">
+      <c r="G4" s="73"/>
+      <c r="H4" s="73"/>
+      <c r="I4" s="74" t="s">
         <v>45</v>
       </c>
-      <c r="J4" s="49"/>
-      <c r="K4" s="49"/>
+      <c r="J4" s="73"/>
+      <c r="K4" s="73"/>
     </row>
     <row r="5" spans="2:11" ht="14.5" x14ac:dyDescent="0.35">
       <c r="B5" s="2" t="s">
@@ -2587,33 +2565,33 @@
       <c r="B6" s="8" t="s">
         <v>63</v>
       </c>
-      <c r="C6" s="39">
+      <c r="C6" s="37">
         <v>0.05</v>
       </c>
-      <c r="D6" s="40">
+      <c r="D6" s="38">
         <v>0.4</v>
       </c>
-      <c r="E6" s="46">
+      <c r="E6" s="44">
         <f t="shared" ref="E6:E8" si="0">D6*C6</f>
         <v>2.0000000000000004E-2</v>
       </c>
-      <c r="F6" s="39">
+      <c r="F6" s="37">
         <v>0.08</v>
       </c>
-      <c r="G6" s="40">
+      <c r="G6" s="38">
         <v>0.7</v>
       </c>
-      <c r="H6" s="46">
+      <c r="H6" s="44">
         <f t="shared" ref="H6:H8" si="1">F6*G6</f>
         <v>5.5999999999999994E-2</v>
       </c>
-      <c r="I6" s="39">
+      <c r="I6" s="37">
         <v>0.08</v>
       </c>
-      <c r="J6" s="40">
+      <c r="J6" s="38">
         <v>0.7</v>
       </c>
-      <c r="K6" s="46">
+      <c r="K6" s="44">
         <f t="shared" ref="K6:K8" si="2">I6*J6</f>
         <v>5.5999999999999994E-2</v>
       </c>
@@ -2622,33 +2600,33 @@
       <c r="B7" s="10" t="s">
         <v>81</v>
       </c>
-      <c r="C7" s="41">
+      <c r="C7" s="39">
         <v>0.06</v>
       </c>
-      <c r="D7" s="42">
+      <c r="D7" s="40">
         <v>0.5</v>
       </c>
-      <c r="E7" s="47">
+      <c r="E7" s="45">
         <f t="shared" si="0"/>
         <v>0.03</v>
       </c>
-      <c r="F7" s="41">
+      <c r="F7" s="39">
         <v>0.1</v>
       </c>
-      <c r="G7" s="42">
+      <c r="G7" s="40">
         <v>0.8</v>
       </c>
-      <c r="H7" s="47">
+      <c r="H7" s="45">
         <f t="shared" si="1"/>
         <v>8.0000000000000016E-2</v>
       </c>
-      <c r="I7" s="41">
+      <c r="I7" s="39">
         <v>0.1</v>
       </c>
-      <c r="J7" s="42">
+      <c r="J7" s="40">
         <v>0.8</v>
       </c>
-      <c r="K7" s="47">
+      <c r="K7" s="45">
         <f t="shared" si="2"/>
         <v>8.0000000000000016E-2</v>
       </c>
@@ -2657,50 +2635,50 @@
       <c r="B8" s="10" t="s">
         <v>87</v>
       </c>
-      <c r="C8" s="41">
+      <c r="C8" s="39">
         <v>0.08</v>
       </c>
-      <c r="D8" s="42">
+      <c r="D8" s="40">
         <v>0.6</v>
       </c>
-      <c r="E8" s="47">
+      <c r="E8" s="45">
         <f t="shared" si="0"/>
         <v>4.8000000000000001E-2</v>
       </c>
-      <c r="F8" s="41">
+      <c r="F8" s="39">
         <v>0.14000000000000001</v>
       </c>
-      <c r="G8" s="42">
+      <c r="G8" s="40">
         <v>0.85</v>
       </c>
-      <c r="H8" s="47">
+      <c r="H8" s="45">
         <f t="shared" si="1"/>
         <v>0.11900000000000001</v>
       </c>
-      <c r="I8" s="41">
+      <c r="I8" s="39">
         <v>0.14000000000000001</v>
       </c>
-      <c r="J8" s="42">
+      <c r="J8" s="40">
         <v>0.85</v>
       </c>
-      <c r="K8" s="47">
+      <c r="K8" s="45">
         <f t="shared" si="2"/>
         <v>0.11900000000000001</v>
       </c>
     </row>
     <row r="10" spans="2:11" ht="48" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B10" s="51" t="s">
+      <c r="B10" s="75" t="s">
         <v>94</v>
       </c>
-      <c r="C10" s="49"/>
-      <c r="D10" s="49"/>
-      <c r="E10" s="49"/>
-      <c r="F10" s="49"/>
-      <c r="G10" s="49"/>
-      <c r="H10" s="49"/>
-      <c r="I10" s="49"/>
-      <c r="J10" s="49"/>
-      <c r="K10" s="49"/>
+      <c r="C10" s="73"/>
+      <c r="D10" s="73"/>
+      <c r="E10" s="73"/>
+      <c r="F10" s="73"/>
+      <c r="G10" s="73"/>
+      <c r="H10" s="73"/>
+      <c r="I10" s="73"/>
+      <c r="J10" s="73"/>
+      <c r="K10" s="73"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -2742,12 +2720,12 @@
       </c>
     </row>
     <row r="3" spans="2:10" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B3" s="55" t="s">
+      <c r="B3" s="79" t="s">
         <v>30</v>
       </c>
-      <c r="C3" s="53"/>
-      <c r="D3" s="53"/>
-      <c r="E3" s="54"/>
+      <c r="C3" s="77"/>
+      <c r="D3" s="77"/>
+      <c r="E3" s="78"/>
     </row>
     <row r="4" spans="2:10" ht="14.5" x14ac:dyDescent="0.35">
       <c r="B4" s="16" t="s">
@@ -2845,11 +2823,11 @@
         <v>91</v>
       </c>
       <c r="C9" s="7">
-        <f>Inputs!$C$12*Inputs!$C$7/100</f>
+        <f>Inputs!$C$11*Inputs!$C$7/100</f>
         <v>43.2</v>
       </c>
       <c r="D9" s="7">
-        <f>Inputs!$C$12</f>
+        <f>Inputs!$C$11</f>
         <v>72</v>
       </c>
       <c r="E9" s="9">
@@ -2865,11 +2843,11 @@
         <v>93</v>
       </c>
       <c r="C10" s="7">
+        <f>Inputs!C12*Inputs!C3</f>
+        <v>510</v>
+      </c>
+      <c r="D10" s="7">
         <f>Inputs!C13*Inputs!C3</f>
-        <v>510</v>
-      </c>
-      <c r="D10" s="7">
-        <f>Inputs!C14*Inputs!C3</f>
         <v>240</v>
       </c>
       <c r="E10" s="9">
@@ -2881,18 +2859,18 @@
       </c>
     </row>
     <row r="11" spans="2:10" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="B11" s="86" t="s">
+      <c r="B11" s="69" t="s">
         <v>96</v>
       </c>
-      <c r="C11" s="87">
-        <f>Inputs!$C$15</f>
+      <c r="C11" s="70">
+        <f>Inputs!$C$14</f>
         <v>0</v>
       </c>
-      <c r="D11" s="87">
+      <c r="D11" s="70">
         <f>C11</f>
         <v>0</v>
       </c>
-      <c r="E11" s="88">
+      <c r="E11" s="71">
         <f>C11</f>
         <v>0</v>
       </c>
@@ -2900,10 +2878,10 @@
     </row>
     <row r="12" spans="2:10" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B12" s="12" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="C12" s="13">
-        <f>Inputs!C16</f>
+        <f>Inputs!C15</f>
         <v>0</v>
       </c>
       <c r="D12" s="13">
@@ -2915,12 +2893,12 @@
     </row>
     <row r="13" spans="2:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="14" spans="2:10" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B14" s="55" t="s">
+      <c r="B14" s="79" t="s">
         <v>97</v>
       </c>
-      <c r="C14" s="53"/>
-      <c r="D14" s="53"/>
-      <c r="E14" s="54"/>
+      <c r="C14" s="77"/>
+      <c r="D14" s="77"/>
+      <c r="E14" s="78"/>
     </row>
     <row r="15" spans="2:10" ht="14.5" x14ac:dyDescent="0.35">
       <c r="B15" s="16" t="s">
@@ -2955,37 +2933,37 @@
         <f t="shared" si="2"/>
         <v>5.0500000000000003E-2</v>
       </c>
-      <c r="F16" s="56" t="s">
+      <c r="F16" s="80" t="s">
         <v>100</v>
       </c>
-      <c r="G16" s="57"/>
-      <c r="H16" s="57"/>
-      <c r="I16" s="57"/>
-      <c r="J16" s="57"/>
+      <c r="G16" s="81"/>
+      <c r="H16" s="81"/>
+      <c r="I16" s="81"/>
+      <c r="J16" s="81"/>
     </row>
     <row r="17" spans="2:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="18" spans="2:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B18" s="55" t="s">
+      <c r="B18" s="79" t="s">
         <v>101</v>
       </c>
-      <c r="C18" s="53"/>
-      <c r="D18" s="53"/>
-      <c r="E18" s="54"/>
+      <c r="C18" s="77"/>
+      <c r="D18" s="77"/>
+      <c r="E18" s="78"/>
     </row>
     <row r="19" spans="2:10" ht="27" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B19" s="58" t="s">
+      <c r="B19" s="82" t="s">
         <v>102</v>
       </c>
-      <c r="C19" s="59"/>
-      <c r="D19" s="59"/>
-      <c r="E19" s="60"/>
-      <c r="F19" s="56" t="s">
+      <c r="C19" s="83"/>
+      <c r="D19" s="83"/>
+      <c r="E19" s="84"/>
+      <c r="F19" s="80" t="s">
         <v>103</v>
       </c>
-      <c r="G19" s="57"/>
-      <c r="H19" s="57"/>
-      <c r="I19" s="57"/>
-      <c r="J19" s="57"/>
+      <c r="G19" s="81"/>
+      <c r="H19" s="81"/>
+      <c r="I19" s="81"/>
+      <c r="J19" s="81"/>
     </row>
     <row r="20" spans="2:10" ht="14.5" x14ac:dyDescent="0.35">
       <c r="B20" s="16" t="s">
@@ -3057,12 +3035,12 @@
     </row>
     <row r="24" spans="2:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="25" spans="2:10" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B25" s="58" t="s">
+      <c r="B25" s="82" t="s">
         <v>116</v>
       </c>
-      <c r="C25" s="53"/>
-      <c r="D25" s="53"/>
-      <c r="E25" s="54"/>
+      <c r="C25" s="77"/>
+      <c r="D25" s="77"/>
+      <c r="E25" s="78"/>
     </row>
     <row r="26" spans="2:10" ht="14.5" x14ac:dyDescent="0.35">
       <c r="B26" s="16" t="s">
@@ -3119,21 +3097,21 @@
       <c r="B29" s="12" t="s">
         <v>112</v>
       </c>
-      <c r="C29" s="61" t="str">
+      <c r="C29" s="85" t="str">
         <f>IF(C28&gt;0,"Year 1",IF(D28&gt;0,"Year 2",IF(E28&gt;0,"Year 3","Beyond Year 3")))</f>
         <v>Year 2</v>
       </c>
-      <c r="D29" s="61"/>
-      <c r="E29" s="62"/>
+      <c r="D29" s="85"/>
+      <c r="E29" s="86"/>
     </row>
     <row r="30" spans="2:10" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="31" spans="2:10" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B31" s="58" t="s">
+      <c r="B31" s="82" t="s">
         <v>120</v>
       </c>
-      <c r="C31" s="53"/>
-      <c r="D31" s="53"/>
-      <c r="E31" s="54"/>
+      <c r="C31" s="77"/>
+      <c r="D31" s="77"/>
+      <c r="E31" s="78"/>
     </row>
     <row r="32" spans="2:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B32" s="16" t="s">
@@ -3190,40 +3168,40 @@
       <c r="B35" s="12" t="s">
         <v>112</v>
       </c>
-      <c r="C35" s="61" t="str">
+      <c r="C35" s="85" t="str">
         <f>IF(C34&gt;0,"Year 1",IF(D34&gt;0,"Year 2",IF(E34&gt;0,"Year 3","Beyond Year 3")))</f>
         <v>Year 2</v>
       </c>
-      <c r="D35" s="61"/>
-      <c r="E35" s="62"/>
+      <c r="D35" s="85"/>
+      <c r="E35" s="86"/>
     </row>
     <row r="36" spans="2:6" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="37" spans="2:6" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B37" s="55" t="s">
+      <c r="B37" s="79" t="s">
         <v>121</v>
       </c>
-      <c r="C37" s="53"/>
-      <c r="D37" s="53"/>
-      <c r="E37" s="54"/>
+      <c r="C37" s="77"/>
+      <c r="D37" s="77"/>
+      <c r="E37" s="78"/>
     </row>
     <row r="38" spans="2:6" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="39" spans="2:6" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B39" s="52" t="s">
+      <c r="B39" s="76" t="s">
         <v>122</v>
       </c>
-      <c r="C39" s="53"/>
-      <c r="D39" s="53"/>
-      <c r="E39" s="54"/>
+      <c r="C39" s="77"/>
+      <c r="D39" s="77"/>
+      <c r="E39" s="78"/>
     </row>
     <row r="40" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B40" s="16"/>
-      <c r="C40" s="37">
+      <c r="C40" s="35">
         <v>0.3</v>
       </c>
-      <c r="D40" s="37">
+      <c r="D40" s="35">
         <v>0.5</v>
       </c>
-      <c r="E40" s="38">
+      <c r="E40" s="36">
         <v>0.7</v>
       </c>
     </row>
@@ -3245,43 +3223,43 @@
       </c>
     </row>
     <row r="42" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B42" s="23" t="s">
+      <c r="B42" s="21" t="s">
         <v>124</v>
       </c>
-      <c r="C42" s="24">
+      <c r="C42" s="22">
         <f>$C$28+($C$5*Scenarios!$F$7*C40-$D$15)</f>
         <v>-2228.3999999999996</v>
       </c>
-      <c r="D42" s="24">
+      <c r="D42" s="22">
         <f>$C$28+($C$5*Scenarios!$F$7*D40-$D$15)</f>
         <v>-1268.3999999999996</v>
       </c>
-      <c r="E42" s="25">
+      <c r="E42" s="23">
         <f>$C$28+($C$5*Scenarios!$F$7*E40-$D$15)</f>
         <v>-308.39999999999964</v>
       </c>
     </row>
     <row r="43" spans="2:6" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4"/>
     <row r="44" spans="2:6" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B44" s="52" t="s">
+      <c r="B44" s="76" t="s">
         <v>125</v>
       </c>
-      <c r="C44" s="53"/>
-      <c r="D44" s="53"/>
-      <c r="E44" s="54"/>
+      <c r="C44" s="77"/>
+      <c r="D44" s="77"/>
+      <c r="E44" s="78"/>
       <c r="F44" s="11" t="s">
         <v>126</v>
       </c>
     </row>
     <row r="45" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B45" s="16"/>
-      <c r="C45" s="43">
+      <c r="C45" s="41">
         <v>500</v>
       </c>
-      <c r="D45" s="43">
+      <c r="D45" s="41">
         <v>600</v>
       </c>
-      <c r="E45" s="44">
+      <c r="E45" s="42">
         <v>800</v>
       </c>
     </row>
@@ -3303,7 +3281,7 @@
       </c>
     </row>
     <row r="47" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B47" s="26" t="s">
+      <c r="B47" s="24" t="s">
         <v>124</v>
       </c>
       <c r="C47" s="15">
@@ -3314,24 +3292,24 @@
         <f t="shared" si="10"/>
         <v>-749.99999999999875</v>
       </c>
-      <c r="E47" s="27">
+      <c r="E47" s="25">
         <f t="shared" si="10"/>
         <v>-1671.5999999999988</v>
       </c>
     </row>
     <row r="48" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B48" s="23" t="s">
+      <c r="B48" s="21" t="s">
         <v>112</v>
       </c>
-      <c r="C48" s="24" t="str">
+      <c r="C48" s="22" t="str">
         <f t="shared" ref="C48:E48" si="11">IF($C$28-$C$8*(C45/400-1)&gt;=0,"Year 1",IF($D$28-($C$8+$D$8)*(C45/400-1)&gt;=0,"Year 2",IF($E$28-($C$8+$D$8+$E$8)*(C45/400-1)&gt;=0,"Year 3","Beyond Year 3")))</f>
         <v>Year 3</v>
       </c>
-      <c r="D48" s="24" t="str">
+      <c r="D48" s="22" t="str">
         <f t="shared" si="11"/>
         <v>Year 3</v>
       </c>
-      <c r="E48" s="25" t="str">
+      <c r="E48" s="23" t="str">
         <f t="shared" si="11"/>
         <v>Beyond Year 3</v>
       </c>
@@ -3362,101 +3340,109 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="B2:G8"/>
+  <dimension ref="B2:G10"/>
   <sheetFormatPr defaultColWidth="14.453125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="47.26953125" customWidth="1"/>
-    <col min="4" max="4" width="51.81640625" customWidth="1"/>
+    <col min="1" max="1" width="14.453125" style="43"/>
+    <col min="2" max="2" width="47.26953125" style="43" customWidth="1"/>
+    <col min="3" max="3" width="14.453125" style="43"/>
+    <col min="4" max="4" width="51.81640625" style="43" customWidth="1"/>
+    <col min="5" max="16384" width="14.453125" style="43"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B2" s="21" t="s">
+      <c r="B2" s="87" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="3" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B3" s="21" t="s">
+      <c r="B3" s="87" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="5" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B5" s="21" t="s">
+      <c r="B5" s="87" t="s">
         <v>109</v>
       </c>
-      <c r="C5" s="22">
+      <c r="C5" s="88">
         <f>Model!D5*Scenarios!F7</f>
         <v>4800</v>
       </c>
-      <c r="D5" s="21" t="s">
+      <c r="D5" s="87" t="s">
         <v>111</v>
       </c>
-      <c r="F5" s="21">
+      <c r="F5" s="87">
         <f>0</f>
         <v>0</v>
       </c>
-      <c r="G5" s="22">
+      <c r="G5" s="88">
         <f>C5</f>
         <v>4800</v>
       </c>
     </row>
     <row r="6" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B6" s="21" t="s">
+      <c r="B6" s="87" t="s">
         <v>113</v>
       </c>
-      <c r="C6" s="22">
+      <c r="C6" s="88">
         <f>-Model!D5*Scenarios!F7*(1-Scenarios!G7)</f>
         <v>-959.99999999999977</v>
       </c>
-      <c r="D6" s="21" t="s">
+      <c r="D6" s="87" t="s">
         <v>114</v>
       </c>
-      <c r="F6" s="22">
+      <c r="F6" s="88">
         <f>C5+C6</f>
         <v>3840</v>
       </c>
-      <c r="G6" s="22">
+      <c r="G6" s="88">
         <f t="shared" ref="G6:G7" si="0">-C6</f>
         <v>959.99999999999977</v>
       </c>
     </row>
     <row r="7" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B7" s="21" t="s">
+      <c r="B7" s="87" t="s">
         <v>115</v>
       </c>
-      <c r="C7" s="22">
+      <c r="C7" s="88">
         <f>-Model!D15</f>
         <v>-2424</v>
       </c>
-      <c r="D7" s="21" t="s">
+      <c r="D7" s="87" t="s">
         <v>117</v>
       </c>
-      <c r="F7" s="22">
+      <c r="F7" s="88">
         <f>F6+C7</f>
         <v>1416</v>
       </c>
-      <c r="G7" s="22">
+      <c r="G7" s="88">
         <f t="shared" si="0"/>
         <v>2424</v>
       </c>
     </row>
     <row r="8" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B8" s="21" t="s">
+      <c r="B8" s="87" t="s">
         <v>118</v>
       </c>
-      <c r="C8" s="22">
+      <c r="C8" s="88">
         <f>SUM(C5:C7)</f>
         <v>1416</v>
       </c>
-      <c r="D8" s="21" t="s">
+      <c r="D8" s="87" t="s">
         <v>119</v>
       </c>
-      <c r="F8" s="21">
+      <c r="F8" s="87">
         <f>0</f>
         <v>0</v>
       </c>
-      <c r="G8" s="22">
+      <c r="G8" s="88">
         <f>C8</f>
         <v>1416</v>
+      </c>
+    </row>
+    <row r="10" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B10" s="43" t="s">
+        <v>152</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Review fix batch: 2.4% tooling figure, Low-scenario sentence, DORA population wording, making-of pointers
</commit_message>
<xml_diff>
--- a/AI_Business_Case_Model.xlsx
+++ b/AI_Business_Case_Model.xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="154">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="179" uniqueCount="156">
   <si>
     <t>AI business case model</t>
   </si>
@@ -508,6 +508,12 @@
   </si>
   <si>
     <t>The monthly cost of the AI-specific platform layer.</t>
+  </si>
+  <si>
+    <t>Authorship</t>
+  </si>
+  <si>
+    <t>The playbook's closing section, How this playbook was made, covers the authorship and composition of the whole set.</t>
   </si>
 </sst>
 </file>
@@ -2153,9 +2159,13 @@
       <c r="B27" s="34"/>
       <c r="C27" s="34"/>
     </row>
-    <row r="28" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B28" s="34"/>
-      <c r="C28" s="34"/>
+    <row r="28" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B28" s="26" t="s">
+        <v>154</v>
+      </c>
+      <c r="C28" s="27" t="s">
+        <v>155</v>
+      </c>
     </row>
     <row r="29" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B29" s="34"/>

</xml_diff>